<commit_message>
@ suppression colonnes A/B/C feuilles Excel: tableau en A-D, module affiche une fois, templates xlsx
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
@
</commit_message>
<xml_diff>
--- a/Templates/METROLOGO_Tachy.xlsx
+++ b/Templates/METROLOGO_Tachy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GLB\Desktop\projet\MetrologoWPF\MetrologoWPF\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD865B17-7FDA-40F0-AB80-54C403552D27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A68B438-20BC-49CD-9318-354F0167A2B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{05031086-6F6F-4E7A-BF9B-F73FC503154F}"/>
+    <workbookView xWindow="3660" yWindow="2610" windowWidth="26685" windowHeight="14085" xr2:uid="{05031086-6F6F-4E7A-BF9B-F73FC503154F}"/>
   </bookViews>
   <sheets>
     <sheet name="ModFeuille" sheetId="1" r:id="rId1"/>
@@ -44,60 +44,60 @@
     <definedName name="_F_Avant_IntervZNPlageFReelle">#REF!</definedName>
     <definedName name="_F_FinaleZNDeltaF">#REF!</definedName>
     <definedName name="_F_FinaleZNPlageFReelle">#REF!</definedName>
-    <definedName name="ZNCoeffA">ModFeuille!$J$2</definedName>
+    <definedName name="ZNCoeffA">ModFeuille!$G$2</definedName>
     <definedName name="ZNCoeffADerive">#REF!</definedName>
-    <definedName name="ZNCoeffB">ModFeuille!$J$3</definedName>
+    <definedName name="ZNCoeffB">ModFeuille!$G$3</definedName>
     <definedName name="ZNCoeffBDerive">#REF!</definedName>
-    <definedName name="ZNCoeffC">ModFeuille!$L$2</definedName>
-    <definedName name="ZNCoeffD">ModFeuille!$L$3</definedName>
+    <definedName name="ZNCoeffC">ModFeuille!$I$2</definedName>
+    <definedName name="ZNCoeffD">ModFeuille!$I$3</definedName>
     <definedName name="ZNCoeffDeriveJournaliere">#REF!</definedName>
-    <definedName name="ZNCoeffMult">ModFeuille!$G$4</definedName>
-    <definedName name="ZNCoeffNbMes">ModFeuille!$J$7</definedName>
-    <definedName name="ZNCoeffTempsMesure">ModFeuille!$J$8</definedName>
+    <definedName name="ZNCoeffMult">ModFeuille!$D$4</definedName>
+    <definedName name="ZNCoeffNbMes">ModFeuille!$G$7</definedName>
+    <definedName name="ZNCoeffTempsMesure">ModFeuille!$G$8</definedName>
     <definedName name="ZNCyclesDerive">#REF!</definedName>
-    <definedName name="ZNDate">ModFeuille!$F$1</definedName>
+    <definedName name="ZNDate">ModFeuille!$C$1</definedName>
     <definedName name="ZNDateRecapDerive">#REF!</definedName>
     <definedName name="ZNDateRecapFreq">'Récap.'!$D$1</definedName>
     <definedName name="ZNDateRecapStab">#REF!</definedName>
     <definedName name="ZNDeriveJournaliere">#REF!</definedName>
-    <definedName name="ZNEcartType">ModFeuille!$F$17</definedName>
-    <definedName name="ZNFNominale">ModFeuille!$F$5</definedName>
-    <definedName name="ZNFreqCorr">ModFeuille!$F$23</definedName>
+    <definedName name="ZNEcartType">ModFeuille!$C$17</definedName>
+    <definedName name="ZNFNominale">ModFeuille!$C$5</definedName>
+    <definedName name="ZNFreqCorr">ModFeuille!$C$23</definedName>
     <definedName name="ZNFreqLisseeDerive">#REF!</definedName>
-    <definedName name="ZNFreqMoyReel">ModFeuille!$F$13</definedName>
-    <definedName name="ZNFreqRef">ModFeuille!$F$21</definedName>
+    <definedName name="ZNFreqMoyReel">ModFeuille!$C$13</definedName>
+    <definedName name="ZNFreqRef">ModFeuille!$C$21</definedName>
     <definedName name="ZNFrequencesMoyennesDerive">#REF!</definedName>
-    <definedName name="ZNFreqUtilise">ModFeuille!$F$2</definedName>
-    <definedName name="ZNGate">ModFeuille!$F$3</definedName>
+    <definedName name="ZNFreqUtilise">ModFeuille!$C$2</definedName>
+    <definedName name="ZNGate">ModFeuille!$C$3</definedName>
     <definedName name="ZNGrandeValeur">#REF!</definedName>
     <definedName name="ZNGraphe_Datas1">#REF!</definedName>
     <definedName name="ZNGraphe_Datas2">#REF!</definedName>
     <definedName name="ZNGraphe_LibsAxeX">#REF!</definedName>
     <definedName name="ZNGraphe_LibSerie1">#REF!</definedName>
     <definedName name="ZNGraphe_LibSerie2">#REF!</definedName>
-    <definedName name="ZNIncertAccreditee">ModFeuille!$F$29</definedName>
-    <definedName name="ZNIncertEcartType">ModFeuille!$F$19</definedName>
-    <definedName name="ZNIncertGlobale">ModFeuille!$F$31</definedName>
-    <definedName name="ZNIncertGlobNONStab">ModFeuille!$J$9</definedName>
+    <definedName name="ZNIncertAccreditee">ModFeuille!$C$29</definedName>
+    <definedName name="ZNIncertEcartType">ModFeuille!$C$19</definedName>
+    <definedName name="ZNIncertGlobale">ModFeuille!$C$31</definedName>
+    <definedName name="ZNIncertGlobNONStab">ModFeuille!$G$9</definedName>
     <definedName name="ZNIncertRecapDerive">#REF!</definedName>
-    <definedName name="ZNIncertResol">ModFeuille!$F$25</definedName>
-    <definedName name="ZNIncertResolRpm">ModFeuille!$I$25</definedName>
-    <definedName name="ZNIncertSup">ModFeuille!$F$27</definedName>
+    <definedName name="ZNIncertResol">ModFeuille!$C$25</definedName>
+    <definedName name="ZNIncertResolRpm">ModFeuille!$F$25</definedName>
+    <definedName name="ZNIncertSup">ModFeuille!$C$27</definedName>
     <definedName name="ZNInfosFinales">#REF!</definedName>
-    <definedName name="ZNLibGate">ModFeuille!$G$3</definedName>
+    <definedName name="ZNLibGate">ModFeuille!$D$3</definedName>
     <definedName name="ZNMaxFreqDerive">#REF!</definedName>
     <definedName name="ZNMesure1">ModFeuille!$9:$9</definedName>
     <definedName name="ZNMesure2">ModFeuille!$10:$10</definedName>
     <definedName name="ZNMinFreqDerive">#REF!</definedName>
-    <definedName name="ZNModeMesure">ModFeuille!$F$4</definedName>
-    <definedName name="ZNNbMesAccredite">ModFeuille!$J$5</definedName>
-    <definedName name="ZNNbMesures">ModFeuille!$D$5</definedName>
-    <definedName name="ZNNoFiche">ModFeuille!$E$1</definedName>
+    <definedName name="ZNModeMesure">ModFeuille!$C$4</definedName>
+    <definedName name="ZNNbMesAccredite">ModFeuille!$G$5</definedName>
+    <definedName name="ZNNbMesures">ModFeuille!$A$5</definedName>
+    <definedName name="ZNNoFiche">ModFeuille!$B$1</definedName>
     <definedName name="ZNNoFicheRecapDerive">#REF!</definedName>
     <definedName name="ZNNoFicheRecapFreq">'Récap.'!$B$1</definedName>
     <definedName name="ZNNoFicheRecapStab">#REF!</definedName>
     <definedName name="ZNPetiteValeur">#REF!</definedName>
-    <definedName name="ZNPointInsertion">ModFeuille!$D$11</definedName>
+    <definedName name="ZNPointInsertion">ModFeuille!$A$11</definedName>
     <definedName name="ZNRecapD_DebZone">#REF!</definedName>
     <definedName name="ZNRecapD_Ligne0">#REF!</definedName>
     <definedName name="ZNRecapD_NbMesCycle">#REF!</definedName>
@@ -108,12 +108,12 @@
     <definedName name="ZNRecapF_NbMes">'Récap.'!$D$3</definedName>
     <definedName name="ZNRecapS_DebZone">#REF!</definedName>
     <definedName name="ZNRecapS_Ligne0">#REF!</definedName>
-    <definedName name="ZNRubidium">ModFeuille!$E$3</definedName>
-    <definedName name="ZNTempsMesureAccredite">ModFeuille!$J$6</definedName>
-    <definedName name="ZNTypeMesure">ModFeuille!$D$2</definedName>
-    <definedName name="ZNValFNominale">ModFeuille!$G$5</definedName>
-    <definedName name="ZNValGateSecondes">ModFeuille!$J$4</definedName>
-    <definedName name="ZNVariance">ModFeuille!$F$15</definedName>
+    <definedName name="ZNRubidium">ModFeuille!$B$3</definedName>
+    <definedName name="ZNTempsMesureAccredite">ModFeuille!$G$6</definedName>
+    <definedName name="ZNTypeMesure">ModFeuille!$A$2</definedName>
+    <definedName name="ZNValFNominale">ModFeuille!$D$5</definedName>
+    <definedName name="ZNValGateSecondes">ModFeuille!$G$4</definedName>
+    <definedName name="ZNVariance">ModFeuille!$C$15</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -133,7 +133,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="44">
   <si>
     <t>HEURE</t>
   </si>
@@ -249,15 +249,6 @@
     <t>Le 31/03/2026</t>
   </si>
   <si>
-    <t>N°Module</t>
-  </si>
-  <si>
-    <t>Fonction</t>
-  </si>
-  <si>
-    <t>Condition 1 (temps de mesure)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Vitesse Moy Réel (RPM) = </t>
   </si>
   <si>
@@ -271,6 +262,9 @@
   </si>
   <si>
     <t>Incert. Globale (RPM) =</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Module = </t>
   </si>
 </sst>
 </file>
@@ -823,255 +817,246 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0A12DF9-E018-409C-98EF-8EE6989ECA7A}">
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" style="1"/>
-    <col min="2" max="2" width="8.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" style="1" customWidth="1"/>
-    <col min="5" max="6" width="25.7109375" style="3" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" style="4" customWidth="1"/>
-    <col min="8" max="8" width="24.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="27.42578125" style="36" customWidth="1"/>
-    <col min="10" max="10" width="23" style="26" customWidth="1"/>
-    <col min="11" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="11.7109375" style="1" customWidth="1"/>
+    <col min="2" max="3" width="25.7109375" style="3" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" style="4" customWidth="1"/>
+    <col min="5" max="5" width="24.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.42578125" style="36" customWidth="1"/>
+    <col min="7" max="7" width="23" style="26" customWidth="1"/>
+    <col min="8" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="D1" s="15" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="2"/>
-      <c r="F1" s="1"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="D2" s="2"/>
-      <c r="F2" s="22"/>
-      <c r="I2" s="36" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" s="2"/>
+      <c r="C2" s="22"/>
+      <c r="F2" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="D3" s="2" t="s">
+      <c r="H2" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="22"/>
-      <c r="F3" s="40"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="41"/>
-      <c r="I3" s="36" t="s">
+      <c r="B3" s="22"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="H3" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C4" s="27"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="37" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" s="28"/>
+      <c r="B5" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="27"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="38" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="F6" s="36" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" s="18"/>
+      <c r="F7" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="26">
+        <f>IF(ISBLANK(ZNNbMesures),,SQRT(ZNNbMesures/ZNNbMesAccredite))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="F8" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="G8" s="26">
+        <f>IF(ISBLANK(ZNValGateSecondes),,ZNTempsMesureAccredite/ZNValGateSecondes)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9" s="19"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="21">
+        <f>IF(ISBLANK(ZNCoeffMult),B9,(((B9-10000000)/(POWER(10,ZNCoeffMult)*10000000))+1)*ZNValFNominale)</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="39" t="s">
+        <v>35</v>
+      </c>
+      <c r="G9" s="26">
+        <f>IF(ISBLANK(ZNIncertSup),,([1]!Cal_incert_global(ZNIncertAccreditee,ZNCoeffNbMes,ZNCoeffTempsMesure,ZNVariance,ZNIncertResol/ZNFreqMoyReel,ZNIncertSup)*ZNFreqMoyReel))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10" s="19"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21">
+        <f>IF(ISBLANK(ZNCoeffMult),B10,(((B10-10000000)/(POWER(10,ZNCoeffMult)*10000000))+1)*ZNValFNominale)</f>
+        <v>0</v>
+      </c>
+      <c r="D10" s="26">
+        <f>C9-C10</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="36" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="F4" s="27"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="28"/>
-      <c r="I4" s="37" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="D5" s="28"/>
-      <c r="E5" s="22" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="27"/>
-      <c r="G5" s="29"/>
-      <c r="H5" s="29"/>
-      <c r="I5" s="38" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="I6" s="36" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="16" t="s">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B13" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="21"/>
+      <c r="E13" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="D7" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="17" t="s">
-        <v>1</v>
-      </c>
-      <c r="F7" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="G7" s="18" t="s">
-        <v>3</v>
-      </c>
-      <c r="H7" s="18"/>
-      <c r="I7" s="36" t="s">
-        <v>33</v>
-      </c>
-      <c r="J7" s="26">
-        <f>IF(ISBLANK(ZNNbMesures),,SQRT(ZNNbMesures/ZNNbMesAccredite))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="I8" s="36" t="s">
-        <v>34</v>
-      </c>
-      <c r="J8" s="26">
-        <f>IF(ISBLANK(ZNValGateSecondes),,ZNTempsMesureAccredite/ZNValGateSecondes)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="D9" s="19"/>
-      <c r="E9" s="21"/>
-      <c r="F9" s="21">
-        <f>IF(ISBLANK(ZNCoeffMult),E9,(((E9-10000000)/(POWER(10,ZNCoeffMult)*10000000))+1)*ZNValFNominale)</f>
-        <v>0</v>
-      </c>
-      <c r="I9" s="39" t="s">
-        <v>35</v>
-      </c>
-      <c r="J9" s="26">
-        <f>IF(ISBLANK(ZNIncertSup),,([1]!Cal_incert_global(ZNIncertAccreditee,ZNCoeffNbMes,ZNCoeffTempsMesure,ZNVariance,ZNIncertResol/ZNFreqMoyReel,ZNIncertSup)*ZNFreqMoyReel))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="D10" s="19"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21">
-        <f>IF(ISBLANK(ZNCoeffMult),E10,(((E10-10000000)/(POWER(10,ZNCoeffMult)*10000000))+1)*ZNValFNominale)</f>
-        <v>0</v>
-      </c>
-      <c r="G10" s="26">
-        <f>F9-F10</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E13" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="F13" s="21"/>
-      <c r="H13" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="I13" s="36">
+      <c r="F13" s="36">
         <f>ZNFreqMoyReel*60</f>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E15" s="3" t="s">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B15" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F15" s="5"/>
-    </row>
-    <row r="17" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E17" s="3" t="s">
+      <c r="C15" s="5"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B17" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F17" s="5">
+      <c r="C17" s="5">
         <f>IF(ISBLANK(ZNVariance),,[1]!Cal_ecart_type(ZNVariance))</f>
         <v>0</v>
       </c>
-      <c r="H17" s="4" t="s">
+      <c r="E17" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="I17" s="36">
+      <c r="F17" s="36">
         <f>ZNEcartType*60</f>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="5:9" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B19" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" s="5">
+        <f>IF(ISBLANK(ZNNbMesures),,[1]!Cal_incert_ecart_type(ZNVariance,ZNNbMesures))</f>
+        <v>0</v>
+      </c>
       <c r="E19" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F19" s="5">
-        <f>IF(ISBLANK(ZNNbMesures),,[1]!Cal_incert_ecart_type(ZNVariance,ZNNbMesures))</f>
-        <v>0</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I19" s="36">
+      <c r="F19" s="36">
         <f>ZNIncertEcartType*60</f>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E21" s="3" t="s">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B21" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F21" s="20"/>
-    </row>
-    <row r="23" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E23" s="3" t="s">
+      <c r="C21" s="20"/>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B23" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="F23" s="20">
+      <c r="C23" s="20">
         <f>IF(ISBLANK(ZNFreqMoyReel),,[1]!Cal_freq_corrigee(ZNFreqMoyReel,ZNFreqRef))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E25" s="3" t="s">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B25" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F25" s="6"/>
-      <c r="H25" s="4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="27" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E27" s="3" t="s">
+      <c r="C25" s="6"/>
+      <c r="E25" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B27" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F27" s="6"/>
-    </row>
-    <row r="29" spans="5:9" x14ac:dyDescent="0.2">
+      <c r="C27" s="6"/>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B29" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29" s="6">
+        <f>IF(ISBLANK(ZNCoeffB),,(IF(ISBLANK(ZNFreqMoyReel),,ZNCoeffB/ZNFreqMoyReel+ZNCoeffA)))</f>
+        <v>0</v>
+      </c>
       <c r="E29" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F29" s="6">
-        <f>IF(ISBLANK(ZNCoeffB),,(IF(ISBLANK(ZNFreqMoyReel),,ZNCoeffB/ZNFreqMoyReel+ZNCoeffA)))</f>
-        <v>0</v>
-      </c>
-      <c r="H29" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I29" s="36">
-        <f>I13*L2+L3</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="5:9" x14ac:dyDescent="0.2">
+      <c r="F29" s="36">
+        <f>F13*I2+I3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B31" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C31" s="6">
+        <f>IF(A2="Stabilité",SQRT(POWER(ZNIncertAccreditee,2)+POWER(ZNIncertEcartType,2)),ZNIncertGlobNONStab)</f>
+        <v>0</v>
+      </c>
       <c r="E31" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F31" s="6">
-        <f>IF(D2="Stabilité",SQRT(POWER(ZNIncertAccreditee,2)+POWER(ZNIncertEcartType,2)),ZNIncertGlobNONStab)</f>
-        <v>0</v>
-      </c>
-      <c r="H31" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="I31" s="36">
-        <f>SQRT(ZNIncertResolRpm^2+I29^2+I17^2+I13^2)</f>
+        <v>42</v>
+      </c>
+      <c r="F31" s="36">
+        <f>SQRT(ZNIncertResolRpm^2+F29^2+F17^2+F13^2)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Template Tachy : mise a jour d une cellule (modif manuelle)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Templates/METROLOGO_Tachy.xlsx
+++ b/Templates/METROLOGO_Tachy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GLB\Desktop\projet\MetrologoWPF\MetrologoWPF\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\G\Desktop\METROLOGO\MetrologoWPF\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A68B438-20BC-49CD-9318-354F0167A2B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{060BC882-5FAF-4CBD-B7E3-425B719ED2C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3660" yWindow="2610" windowWidth="26685" windowHeight="14085" xr2:uid="{05031086-6F6F-4E7A-BF9B-F73FC503154F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{05031086-6F6F-4E7A-BF9B-F73FC503154F}"/>
   </bookViews>
   <sheets>
     <sheet name="ModFeuille" sheetId="1" r:id="rId1"/>
@@ -128,6 +128,9 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -475,9 +478,6 @@
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:relativeUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Feuil1"/>
       <sheetName val="Feuil2"/>
@@ -1056,7 +1056,7 @@
         <v>42</v>
       </c>
       <c r="F31" s="36">
-        <f>SQRT(ZNIncertResolRpm^2+F29^2+F17^2+F13^2)</f>
+        <f>SQRT(ZNIncertResolRpm^2+F29^2+F17^2)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>